<commit_message>
[Feat] AttackRange / AttackArea 분리 (사거리 vs 공격 범위)
- TurretTrainStatus, RangeTrainStatus: AttackArea 필드 추가
  - StatType: AttackArea enum 값 추가
  - TurretTrain: DetectTarget은 AttackRange 유지, projectile 스케일/AoE에 AttackArea 사용
  - TurretTrain: ApplyStat AttackRange case에서 projectile 업데이트 제거, AttackArea case 신규 추가
  - RangeTrain: localScale / Init에 AttackArea 사용, ApplyStat AttackArea case 추가
  - Projectile: _attackRange → _scaleRadius, Init 파라미터명, IsScaleByAttackRange() → IsScaleByArea()
  - ProjectileData: ScaleByRange → ScaleByArea 프로퍼티 리네임
  - ScaleByRangeType: AttackRange → Area 리네임
  - Row 4개: attackArea 필드 및 attack_area 엑셀 매핑 추가
  - Reflector 2개, Importer 4개: AttackArea 반영
  - DatabaseGeneratorWindow: turret/range_train_data 쓰기 로직 전체 스탯 포함으로 개선
  - TriChoiceSelectUI: AttackArea 업그레이드 표시 추가
  - TrainData.xlsx turret/range_train_data: attack_area 컬럼 추가 (attack_range 값 복사)
  - TrainUpgradeData.xlsx turret/range_train_upgrade_data: attack_area 컬럼 추가 (기본값 0)
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainUpgradeData.xlsx
+++ b/Assets/02_Resources/Data/TrainUpgradeData.xlsx
@@ -16,119 +16,122 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="37">
-  <si>
-    <t xml:space="preserve">공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격하는 적 수 &lt;color=#FF5851&gt;&lt;bounce&gt;{1} 증가&lt;/bounce&gt;&lt;/color&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_interval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">critical_damage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_count</t>
-  </si>
-  <si>
-    <t xml:space="preserve">attack_damage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">critical_chance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">upgrade_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">절대무적_요새_288버켓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">절대무적_요새_멜리에스클래식_몸통뉴</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weapon_KMD_08_UI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weapon_MEL_05_UI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weapon_KMD_10_UI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weapon_288_19_UI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">폭발 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">냉기 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격딜레이 &lt;color=#5196FF&gt;&lt;bounce&gt;{1}감소&lt;/bounce&gt;&lt;/color&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 범위 &lt;color=#FF5851&gt;&lt;bounce&gt;{1} 증가&lt;/bounce&gt;&lt;/color&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격 범위 &lt;color=#FF5851&gt;&lt;bounce&gt;{1} 증가&lt;/bounce&gt;&lt;/color&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 &lt;bounce&gt;&lt;color=#FF5851&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격딜레이 &lt;color=#5196FF&gt;&lt;bounce&gt;{1}감소&lt;/bounce&gt;&lt;/color&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격딜레이 &lt;color=#5196FF&gt;&lt;bounce&gt;{1} 감소&lt;/bounce&gt;&lt;/color&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weapon_KMD_12_UI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weapon_MEL_16_UI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weapon_MEL_14_UI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_hp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">icon_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">화염 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미사일 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">레이저 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">포격 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">전기 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">저격 포탑 강화</t>
-  </si>
-  <si>
-    <t xml:space="preserve">target_count</t>
-  </si>
-</sst>
+<ns0:sst xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+  <ns0:si>
+    <ns0:t>공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격하는 적 수 &lt;color=#FF5851&gt;&lt;bounce&gt;{1} 증가&lt;/bounce&gt;&lt;/color&gt;</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>id</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>attack_interval</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>critical_damage</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>attack_range</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>attack_count</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>attack_damage</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>critical_chance</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>upgrade_name</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>절대무적_요새_288버켓</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>절대무적_요새_멜리에스클래식_몸통뉴</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Weapon_KMD_08_UI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Weapon_MEL_05_UI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Weapon_KMD_10_UI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Weapon_288_19_UI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>폭발 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>description</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>냉기 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt;</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격딜레이 &lt;color=#5196FF&gt;&lt;bounce&gt;{1}감소&lt;/bounce&gt;&lt;/color&gt;</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 범위 &lt;color=#FF5851&gt;&lt;bounce&gt;{1} 증가&lt;/bounce&gt;&lt;/color&gt;</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격 범위 &lt;color=#FF5851&gt;&lt;bounce&gt;{1} 증가&lt;/bounce&gt;&lt;/color&gt;</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>공격력 &lt;bounce&gt;&lt;color=#FF5851&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격딜레이 &lt;color=#5196FF&gt;&lt;bounce&gt;{1}감소&lt;/bounce&gt;&lt;/color&gt;</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>공격력 &lt;color=#FF5851&gt;&lt;bounce&gt;{0} 증가&lt;/bounce&gt;&lt;/color&gt; 공격딜레이 &lt;color=#5196FF&gt;&lt;bounce&gt;{1} 감소&lt;/bounce&gt;&lt;/color&gt;</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Weapon_KMD_12_UI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Weapon_MEL_16_UI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>Weapon_MEL_14_UI</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>max_hp</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>icon_id</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>기관총 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>화염 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>미사일 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>레이저 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>포격 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>전기 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>저격 포탑 강화</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>target_count</ns0:t>
+  </ns0:si>
+  <ns0:si>
+    <ns0:t>attack_area</ns0:t>
+  </ns0:si>
+</ns0:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -668,7 +671,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" ns1:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:L8"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.4"/>
@@ -703,16 +706,19 @@
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -735,10 +741,13 @@
       <c r="G2" s="1">
         <v>1</v>
       </c>
-      <c r="J2" s="1">
+      <c r="H2">
         <v>0</v>
       </c>
       <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
         <v>0</v>
       </c>
     </row>
@@ -761,10 +770,13 @@
       <c r="G3" s="1">
         <v>2</v>
       </c>
-      <c r="J3" s="1">
+      <c r="H3">
         <v>0</v>
       </c>
       <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
         <v>0</v>
       </c>
     </row>
@@ -787,10 +799,13 @@
       <c r="G4" s="1">
         <v>4</v>
       </c>
-      <c r="J4" s="1">
+      <c r="H4">
         <v>0</v>
       </c>
       <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
         <v>0</v>
       </c>
     </row>
@@ -813,10 +828,13 @@
       <c r="G5" s="1">
         <v>2</v>
       </c>
-      <c r="J5" s="1">
+      <c r="H5">
         <v>0</v>
       </c>
       <c r="K5" s="1">
+        <v>0</v>
+      </c>
+      <c r="L5" s="1">
         <v>0</v>
       </c>
     </row>
@@ -839,10 +857,13 @@
       <c r="G6" s="1">
         <v>3</v>
       </c>
-      <c r="J6" s="1">
+      <c r="H6">
         <v>0</v>
       </c>
       <c r="K6" s="1">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1">
         <v>0</v>
       </c>
     </row>
@@ -865,16 +886,22 @@
       <c r="G7" s="1">
         <v>4</v>
       </c>
-      <c r="J7" s="1">
+      <c r="H7">
         <v>0</v>
       </c>
       <c r="K7" s="1">
+        <v>0</v>
+      </c>
+      <c r="L7" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="6:7">
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
+      <c r="H8">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -883,7 +910,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" ns1:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:M23"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.4"/>
@@ -920,19 +947,22 @@
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="K1" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -953,14 +983,17 @@
         <v>5</v>
       </c>
       <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1">
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1">
         <v>0.05</v>
       </c>
-      <c r="K2" s="1">
-        <v>0</v>
-      </c>
       <c r="L2" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
         <v>0</v>
       </c>
     </row>
@@ -981,14 +1014,17 @@
         <v>10</v>
       </c>
       <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1">
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1">
         <v>0.05</v>
       </c>
-      <c r="K3" s="1">
-        <v>0</v>
-      </c>
       <c r="L3" s="1">
+        <v>0</v>
+      </c>
+      <c r="M3" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1009,14 +1045,17 @@
         <v>25</v>
       </c>
       <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1">
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1">
         <v>0.05</v>
       </c>
-      <c r="K4" s="1">
-        <v>0</v>
-      </c>
       <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1037,12 +1076,15 @@
         <v>2</v>
       </c>
       <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="H5">
+        <v>0</v>
+      </c>
       <c r="I5" s="1"/>
-      <c r="K5" s="1">
-        <v>0</v>
-      </c>
+      <c r="J5" s="1"/>
       <c r="L5" s="1">
+        <v>0</v>
+      </c>
+      <c r="M5" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1063,12 +1105,15 @@
         <v>3</v>
       </c>
       <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
+      <c r="H6">
+        <v>0</v>
+      </c>
       <c r="I6" s="1"/>
-      <c r="K6" s="1">
-        <v>0</v>
-      </c>
+      <c r="J6" s="1"/>
       <c r="L6" s="1">
+        <v>0</v>
+      </c>
+      <c r="M6" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1089,12 +1134,15 @@
         <v>6</v>
       </c>
       <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
+      <c r="H7">
+        <v>0</v>
+      </c>
       <c r="I7" s="1"/>
-      <c r="K7" s="1">
-        <v>0</v>
-      </c>
+      <c r="J7" s="1"/>
       <c r="L7" s="1">
+        <v>0</v>
+      </c>
+      <c r="M7" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1115,14 +1163,17 @@
         <v>15</v>
       </c>
       <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1">
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1">
         <v>0.14999999999999999</v>
       </c>
-      <c r="K8" s="1">
-        <v>0</v>
-      </c>
       <c r="L8" s="1">
+        <v>0</v>
+      </c>
+      <c r="M8" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1143,14 +1194,17 @@
         <v>20</v>
       </c>
       <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1">
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1">
         <v>0.14999999999999999</v>
       </c>
-      <c r="K9" s="1">
-        <v>0</v>
-      </c>
       <c r="L9" s="1">
+        <v>0</v>
+      </c>
+      <c r="M9" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1171,14 +1225,17 @@
         <v>40</v>
       </c>
       <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1">
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1">
         <v>0.20000000000000001</v>
       </c>
-      <c r="K10" s="1">
-        <v>0</v>
-      </c>
       <c r="L10" s="1">
+        <v>0</v>
+      </c>
+      <c r="M10" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1199,12 +1256,15 @@
         <v>50</v>
       </c>
       <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="H11">
+        <v>0</v>
+      </c>
       <c r="I11" s="1"/>
-      <c r="K11" s="1">
-        <v>0</v>
-      </c>
+      <c r="J11" s="1"/>
       <c r="L11" s="1">
+        <v>0</v>
+      </c>
+      <c r="M11" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1225,12 +1285,15 @@
         <v>50</v>
       </c>
       <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
+      <c r="H12">
+        <v>0</v>
+      </c>
       <c r="I12" s="1"/>
-      <c r="K12" s="1">
-        <v>0</v>
-      </c>
+      <c r="J12" s="1"/>
       <c r="L12" s="1">
+        <v>0</v>
+      </c>
+      <c r="M12" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1251,12 +1314,15 @@
         <v>100</v>
       </c>
       <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
+      <c r="H13">
+        <v>0</v>
+      </c>
       <c r="I13" s="1"/>
-      <c r="K13" s="1">
-        <v>0</v>
-      </c>
+      <c r="J13" s="1"/>
       <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1277,15 +1343,18 @@
         <v>3</v>
       </c>
       <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
+      <c r="H14">
+        <v>0</v>
+      </c>
       <c r="I14" s="1"/>
-      <c r="J14" s="0">
+      <c r="J14" s="1"/>
+      <c r="K14" s="0">
         <v>2</v>
       </c>
-      <c r="K14" s="1">
-        <v>0</v>
-      </c>
       <c r="L14" s="1">
+        <v>0</v>
+      </c>
+      <c r="M14" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1306,15 +1375,18 @@
         <v>5</v>
       </c>
       <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
+      <c r="H15">
+        <v>0</v>
+      </c>
       <c r="I15" s="1"/>
-      <c r="J15" s="0">
+      <c r="J15" s="1"/>
+      <c r="K15" s="0">
         <v>2</v>
       </c>
-      <c r="K15" s="1">
-        <v>0</v>
-      </c>
       <c r="L15" s="1">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1335,15 +1407,18 @@
         <v>7</v>
       </c>
       <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
+      <c r="H16">
+        <v>0</v>
+      </c>
       <c r="I16" s="1"/>
-      <c r="J16" s="0">
+      <c r="J16" s="1"/>
+      <c r="K16" s="0">
         <v>3</v>
       </c>
-      <c r="K16" s="1">
-        <v>0</v>
-      </c>
       <c r="L16" s="1">
+        <v>0</v>
+      </c>
+      <c r="M16" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1366,12 +1441,15 @@
       <c r="G17" s="1">
         <v>1</v>
       </c>
-      <c r="H17" s="1"/>
+      <c r="H17">
+        <v>0</v>
+      </c>
       <c r="I17" s="1"/>
-      <c r="K17" s="1">
-        <v>0</v>
-      </c>
+      <c r="J17" s="1"/>
       <c r="L17" s="1">
+        <v>0</v>
+      </c>
+      <c r="M17" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1394,12 +1472,15 @@
       <c r="G18" s="1">
         <v>2</v>
       </c>
-      <c r="H18" s="1"/>
+      <c r="H18">
+        <v>0</v>
+      </c>
       <c r="I18" s="1"/>
-      <c r="K18" s="1">
-        <v>0</v>
-      </c>
+      <c r="J18" s="1"/>
       <c r="L18" s="1">
+        <v>0</v>
+      </c>
+      <c r="M18" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1422,12 +1503,15 @@
       <c r="G19" s="1">
         <v>4</v>
       </c>
-      <c r="H19" s="1"/>
+      <c r="H19">
+        <v>0</v>
+      </c>
       <c r="I19" s="1"/>
-      <c r="K19" s="1">
-        <v>0</v>
-      </c>
+      <c r="J19" s="1"/>
       <c r="L19" s="1">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1448,14 +1532,17 @@
         <v>50</v>
       </c>
       <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1">
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1">
         <v>0.05</v>
       </c>
-      <c r="K20" s="1">
-        <v>0</v>
-      </c>
       <c r="L20" s="1">
+        <v>0</v>
+      </c>
+      <c r="M20" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1476,14 +1563,17 @@
         <v>75</v>
       </c>
       <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1">
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1">
         <v>0.05</v>
       </c>
-      <c r="K21" s="1">
-        <v>0</v>
-      </c>
       <c r="L21" s="1">
+        <v>0</v>
+      </c>
+      <c r="M21" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1504,22 +1594,28 @@
         <v>125</v>
       </c>
       <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1">
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1">
         <v>0.14999999999999999</v>
       </c>
-      <c r="K22" s="1">
-        <v>0</v>
-      </c>
       <c r="L22" s="1">
+        <v>0</v>
+      </c>
+      <c r="M22" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="6:10">
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
+      <c r="H23">
+        <v>0</v>
+      </c>
       <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>